<commit_message>
Figure S15 and Table S3: three conditions (PITCH, MLP + IG, measurement-only); context-only kept as an unused control
Final decision: the context-only control is not part of Figure S15 or Table S3. Figure S15 data, plotting script and figure are restored to the
three-condition version (data files identical to the earlier version); Table S3 script and outputs show 12 rows (3 conditions x 4 LLMs).
The derived context-only results are removed from the repository (four-condition radars, datasheet, per-model score table, context-only rows in
the agreement summary table). Kept so that a reviewer can inspect and re-run the control: generation, selection and judging scripts (with
--conds cond4_context_only_softened), the exploratory 02h script, 04d --with-context-only, the prompts, answers, verdicts, judge scorecards and
agreement records. Table S2 keeps the generation-rate row of the control. READMEs updated accordingly.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/6_supplementary_figures/TableS3_quality_by_model/TableS3_quality_by_model.xlsx
+++ b/6_supplementary_figures/TableS3_quality_by_model/TableS3_quality_by_model.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -913,154 +913,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Context-only</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Qwen3.8</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>10.00†</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>8.83</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>8.83</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>8.83†</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>8.33</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>DeepSeek</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>9.50†</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>8.50</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>8.50</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>8.33†</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>8.67</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>GLM-5.3</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>8.67†</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>7.50</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>7.83</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>7.17†</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>7.00</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Gemini</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>10.00†</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>8.17</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>7.67</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>7.83†</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>7.17</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1072,7 +924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1099,13 +951,6 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>† Not applicable to Context-only (no focus / contextual features are supplied); shown for reference only.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>